<commit_message>
#40 Item Type added in resistors
</commit_message>
<xml_diff>
--- a/BOM Format/eSpark.Bom.Template.xlsx
+++ b/BOM Format/eSpark.Bom.Template.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\eSpark-Hardware\BOM Format\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\eSpark-Hardware\BOM Format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372D6B6D-320F-49C4-91CF-28C8AE98B74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -88,12 +87,6 @@
     <t>Column=Reviewer Remarks</t>
   </si>
   <si>
-    <t>Column=UnitCost (5 Boards)</t>
-  </si>
-  <si>
-    <t>Column=TotalCost (5 Boards)</t>
-  </si>
-  <si>
     <t>Column=MOQ (5 Boards)</t>
   </si>
   <si>
@@ -104,18 +97,24 @@
   </si>
   <si>
     <t>Single Board Cost</t>
+  </si>
+  <si>
+    <t>Column=Unit Cost (5 Boards)</t>
+  </si>
+  <si>
+    <t>Column=Total Cost (5 Boards)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,6 +255,13 @@
     <font>
       <b/>
       <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -538,7 +544,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -684,6 +690,15 @@
     <xf numFmtId="166" fontId="15" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -716,13 +731,13 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1064,7 +1079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:S14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1100,15 +1115,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="56"/>
+      <c r="K1" s="58"/>
+      <c r="L1" s="58"/>
+      <c r="M1" s="58"/>
+      <c r="N1" s="58"/>
+      <c r="O1" s="58"/>
+      <c r="P1" s="58"/>
+      <c r="Q1" s="58"/>
+      <c r="R1" s="58"/>
+      <c r="S1" s="59"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1158,7 +1173,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="57"/>
+      <c r="S3" s="60"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1183,7 +1198,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="58"/>
+      <c r="S4" s="61"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1208,7 +1223,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="58"/>
+      <c r="S5" s="61"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1229,7 +1244,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="58"/>
+      <c r="S6" s="61"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1250,7 +1265,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="58"/>
+      <c r="S7" s="61"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1271,7 +1286,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="58"/>
+      <c r="S8" s="61"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1309,19 +1324,19 @@
         <v>10</v>
       </c>
       <c r="M9" s="33" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="N9" s="33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O9" s="33" t="s">
         <v>16</v>
       </c>
       <c r="P9" s="33" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="Q9" s="33" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="R9" s="33" t="s">
         <v>17</v>
@@ -1336,7 +1351,7 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="40"/>
+      <c r="C10" s="68"/>
       <c r="D10" s="40"/>
       <c r="E10" s="40"/>
       <c r="F10" s="40"/>
@@ -1358,7 +1373,7 @@
         <v>0</v>
       </c>
       <c r="R10" s="40"/>
-      <c r="S10" s="65"/>
+      <c r="S10" s="55"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
@@ -1366,29 +1381,29 @@
         <f t="shared" ref="B11:B12" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="66"/>
-      <c r="D11" s="66"/>
-      <c r="E11" s="66"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="66"/>
-      <c r="H11" s="66"/>
-      <c r="I11" s="66"/>
-      <c r="J11" s="66"/>
-      <c r="K11" s="66"/>
-      <c r="L11" s="66"/>
-      <c r="M11" s="66">
+      <c r="C11" s="69"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="56"/>
+      <c r="G11" s="56"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="56"/>
+      <c r="J11" s="56"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56">
         <f t="shared" ref="M11:M12" si="1">L11*5</f>
         <v>0</v>
       </c>
-      <c r="N11" s="66"/>
-      <c r="O11" s="66"/>
-      <c r="P11" s="67"/>
-      <c r="Q11" s="67">
+      <c r="N11" s="56"/>
+      <c r="O11" s="56"/>
+      <c r="P11" s="57"/>
+      <c r="Q11" s="57">
         <f t="shared" ref="Q11:Q12" si="2">P11*N11</f>
         <v>0</v>
       </c>
-      <c r="R11" s="66"/>
-      <c r="S11" s="66"/>
+      <c r="R11" s="56"/>
+      <c r="S11" s="56"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -1396,7 +1411,7 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="42"/>
+      <c r="C12" s="70"/>
       <c r="D12" s="42"/>
       <c r="E12" s="42"/>
       <c r="F12" s="42"/>
@@ -1434,17 +1449,17 @@
       <c r="K13" s="49"/>
       <c r="L13" s="49"/>
       <c r="M13" s="49"/>
-      <c r="N13" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="O13" s="64"/>
-      <c r="P13" s="64"/>
+      <c r="N13" s="66" t="s">
+        <v>24</v>
+      </c>
+      <c r="O13" s="67"/>
+      <c r="P13" s="67"/>
       <c r="Q13" s="53" t="e">
         <f>SUM(#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="R13" s="59"/>
-      <c r="S13" s="60"/>
+      <c r="R13" s="62"/>
+      <c r="S13" s="63"/>
     </row>
     <row r="14" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -1460,17 +1475,17 @@
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
-      <c r="N14" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="O14" s="64"/>
-      <c r="P14" s="64"/>
+      <c r="N14" s="66" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" s="67"/>
+      <c r="P14" s="67"/>
       <c r="Q14" s="54" t="e">
         <f>Q13/5</f>
         <v>#REF!</v>
       </c>
-      <c r="R14" s="61"/>
-      <c r="S14" s="62"/>
+      <c r="R14" s="64"/>
+      <c r="S14" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
#30 eSpark BOM template updated.
</commit_message>
<xml_diff>
--- a/BOM Format/eSpark.Bom.Template.xlsx
+++ b/BOM Format/eSpark.Bom.Template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Component list</t>
   </si>
@@ -27,22 +27,10 @@
     <t>Field=Title</t>
   </si>
   <si>
-    <t>Source Data From:</t>
-  </si>
-  <si>
-    <t>Field=DataSourceFileName</t>
-  </si>
-  <si>
     <t>Project:</t>
   </si>
   <si>
     <t>Field=ProjectFileName</t>
-  </si>
-  <si>
-    <t>Variant:</t>
-  </si>
-  <si>
-    <t>Field=VariantName</t>
   </si>
   <si>
     <t>#</t>
@@ -114,7 +102,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,13 +157,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="0"/>
       <name val="Arial"/>
@@ -197,12 +178,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -254,14 +229,22 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -293,7 +276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -320,46 +303,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -422,30 +365,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -544,201 +463,145 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="15" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -768,15 +631,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>10417</xdr:rowOff>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>1724025</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:colOff>1752600</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>161033</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -804,7 +667,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="29927550" y="620017"/>
+          <a:off x="26222325" y="257175"/>
           <a:ext cx="1714500" cy="1104008"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1081,11 +944,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="29" customWidth="1"/>
-    <col min="3" max="3" width="18" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="18" style="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.42578125" customWidth="1"/>
     <col min="5" max="5" width="30.85546875" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
@@ -1096,7 +959,7 @@
     <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.42578125" customWidth="1"/>
+    <col min="14" max="14" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -1106,8 +969,8 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -1115,385 +978,337 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="59"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="46"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="11" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="3"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="38"/>
+      <c r="R2" s="38"/>
+      <c r="S2" s="49"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="13" t="s">
+      <c r="B3" s="8"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="13"/>
-      <c r="F3" s="14" t="s">
+      <c r="E3" s="32"/>
+      <c r="F3" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="60"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="50"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="16"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="61"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
+      <c r="R4" s="29"/>
+      <c r="S4" s="50"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="13" t="s">
+      <c r="B5" s="9"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
+      <c r="S5" s="50"/>
+    </row>
+    <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="41"/>
+      <c r="R6" s="41"/>
+      <c r="S6" s="51"/>
+    </row>
+    <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="L7" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="13"/>
-      <c r="F5" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="18"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="61"/>
+      <c r="M7" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="O7" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="P7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="R7" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="S7" s="12" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="26"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="61"/>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="18">
+        <f>ROW(B8) - ROW($B$7)</f>
+        <v>1</v>
+      </c>
+      <c r="C8" s="26"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14">
+        <f>L8*5</f>
+        <v>0</v>
+      </c>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15">
+        <f>P8*N8</f>
+        <v>0</v>
+      </c>
+      <c r="R8" s="14"/>
+      <c r="S8" s="23"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8"/>
-      <c r="S7" s="61"/>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="19">
+        <f t="shared" ref="B9:B10" si="0">ROW(B9) - ROW($B$7)</f>
+        <v>2</v>
+      </c>
+      <c r="C9" s="27"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24">
+        <f t="shared" ref="M9:M10" si="1">L9*5</f>
+        <v>0</v>
+      </c>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="25">
+        <f t="shared" ref="Q9:Q10" si="2">P9*N9</f>
+        <v>0</v>
+      </c>
+      <c r="R9" s="24"/>
+      <c r="S9" s="24"/>
     </row>
-    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="61"/>
-    </row>
-    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="L9" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="M9" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="N9" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="O9" s="33" t="s">
-        <v>16</v>
-      </c>
-      <c r="P9" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q9" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="R9" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="S9" s="33" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="50">
-        <f>ROW(B10) - ROW($B$9)</f>
-        <v>1</v>
-      </c>
-      <c r="C10" s="68"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40">
-        <f>L10*5</f>
-        <v>0</v>
-      </c>
-      <c r="N10" s="40"/>
-      <c r="O10" s="40"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="41">
-        <f>P10*N10</f>
-        <v>0</v>
-      </c>
-      <c r="R10" s="40"/>
-      <c r="S10" s="55"/>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="51">
-        <f t="shared" ref="B11:B12" si="0">ROW(B11) - ROW($B$9)</f>
-        <v>2</v>
-      </c>
-      <c r="C11" s="69"/>
-      <c r="D11" s="56"/>
-      <c r="E11" s="56"/>
-      <c r="F11" s="56"/>
-      <c r="G11" s="56"/>
-      <c r="H11" s="56"/>
-      <c r="I11" s="56"/>
-      <c r="J11" s="56"/>
-      <c r="K11" s="56"/>
-      <c r="L11" s="56"/>
-      <c r="M11" s="56">
-        <f t="shared" ref="M11:M12" si="1">L11*5</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="56"/>
-      <c r="O11" s="56"/>
-      <c r="P11" s="57"/>
-      <c r="Q11" s="57">
-        <f t="shared" ref="Q11:Q12" si="2">P11*N11</f>
-        <v>0</v>
-      </c>
-      <c r="R11" s="56"/>
-      <c r="S11" s="56"/>
-    </row>
-    <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="52">
+      <c r="B10" s="20">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="70"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="42"/>
-      <c r="M12" s="42">
+      <c r="C10" s="28"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N12" s="42"/>
-      <c r="O12" s="42"/>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="43">
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="R12" s="42"/>
-      <c r="S12" s="42"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="16"/>
     </row>
-    <row r="13" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="44"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="48"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="48"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="48"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="49"/>
-      <c r="M13" s="49"/>
-      <c r="N13" s="66" t="s">
-        <v>24</v>
-      </c>
-      <c r="O13" s="67"/>
-      <c r="P13" s="67"/>
-      <c r="Q13" s="53" t="e">
+    <row r="11" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="O11" s="48"/>
+      <c r="P11" s="48"/>
+      <c r="Q11" s="21" t="e">
         <f>SUM(#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="R13" s="62"/>
-      <c r="S13" s="63"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
     </row>
-    <row r="14" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="66" t="s">
-        <v>25</v>
-      </c>
-      <c r="O14" s="67"/>
-      <c r="P14" s="67"/>
-      <c r="Q14" s="54" t="e">
-        <f>Q13/5</f>
+    <row r="12" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="O12" s="48"/>
+      <c r="P12" s="48"/>
+      <c r="Q12" s="22" t="e">
+        <f>Q11/5</f>
         <v>#REF!</v>
       </c>
-      <c r="R14" s="64"/>
-      <c r="S14" s="65"/>
+      <c r="R12" s="1"/>
+      <c r="S12" s="1"/>
+    </row>
+    <row r="24" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M24" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="K1:S1"/>
-    <mergeCell ref="S3:S8"/>
-    <mergeCell ref="R13:S14"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="N11:P11"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="S2:S6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
#13 eSpark BOM format update
</commit_message>
<xml_diff>
--- a/BOM Format/eSpark.Bom.Template.xlsx
+++ b/BOM Format/eSpark.Bom.Template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Component list</t>
   </si>
@@ -70,9 +70,6 @@
   </si>
   <si>
     <t>Column=Alternate Part Number</t>
-  </si>
-  <si>
-    <t>Column=Reviewer Remarks</t>
   </si>
   <si>
     <t>Column=MOQ (5 Boards)</t>
@@ -102,7 +99,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,13 +122,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color indexed="13"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <color indexed="10"/>
       <name val="Arial"/>
@@ -216,13 +206,6 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -276,7 +259,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -294,42 +277,11 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -408,17 +360,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -463,145 +404,130 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -624,60 +550,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>1752600</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>161033</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="26222325" y="257175"/>
-          <a:ext cx="1714500" cy="1104008"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -944,7 +816,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="10" customWidth="1"/>
@@ -964,10 +836,9 @@
     <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -986,9 +857,8 @@
       <c r="P1" s="45"/>
       <c r="Q1" s="45"/>
       <c r="R1" s="45"/>
-      <c r="S1" s="46"/>
-    </row>
-    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="7"/>
       <c r="C2" s="13"/>
@@ -1001,107 +871,102 @@
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
-      <c r="Q2" s="38"/>
-      <c r="R2" s="38"/>
-      <c r="S2" s="49"/>
-    </row>
-    <row r="3" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I2" s="36"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
+      <c r="R2" s="37"/>
+    </row>
+    <row r="3" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="8"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="52" t="s">
+      <c r="C3" s="30"/>
+      <c r="D3" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="32"/>
-      <c r="F3" s="34" t="s">
+      <c r="E3" s="31"/>
+      <c r="F3" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="29"/>
-      <c r="S3" s="50"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="G3" s="34"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="28"/>
+      <c r="R3" s="28"/>
+    </row>
+    <row r="4" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="8"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="29"/>
-      <c r="R4" s="29"/>
-      <c r="S4" s="50"/>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="C4" s="30"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
+      <c r="R4" s="28"/>
+    </row>
+    <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="9"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="41"/>
-      <c r="N5" s="41"/>
-      <c r="O5" s="41"/>
-      <c r="P5" s="41"/>
-      <c r="Q5" s="41"/>
-      <c r="R5" s="41"/>
-      <c r="S5" s="50"/>
-    </row>
-    <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="38"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+      <c r="L5" s="40"/>
+      <c r="M5" s="40"/>
+      <c r="N5" s="40"/>
+      <c r="O5" s="40"/>
+      <c r="P5" s="40"/>
+      <c r="Q5" s="40"/>
+      <c r="R5" s="40"/>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="41"/>
-      <c r="L6" s="41"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-      <c r="P6" s="41"/>
-      <c r="Q6" s="41"/>
-      <c r="R6" s="41"/>
-      <c r="S6" s="51"/>
-    </row>
-    <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="41"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="40"/>
+      <c r="L6" s="40"/>
+      <c r="M6" s="40"/>
+      <c r="N6" s="40"/>
+      <c r="O6" s="40"/>
+      <c r="P6" s="40"/>
+      <c r="Q6" s="40"/>
+      <c r="R6" s="40"/>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="12" t="s">
         <v>4</v>
@@ -1137,34 +1002,31 @@
         <v>6</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O7" s="12" t="s">
         <v>12</v>
       </c>
       <c r="P7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q7" s="12" t="s">
         <v>22</v>
-      </c>
-      <c r="Q7" s="12" t="s">
-        <v>23</v>
       </c>
       <c r="R7" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="S7" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="18">
         <f>ROW(B8) - ROW($B$7)</f>
         <v>1</v>
       </c>
-      <c r="C8" s="26"/>
+      <c r="C8" s="25"/>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -1186,45 +1048,43 @@
         <v>0</v>
       </c>
       <c r="R8" s="14"/>
-      <c r="S8" s="23"/>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="19">
         <f t="shared" ref="B9:B10" si="0">ROW(B9) - ROW($B$7)</f>
         <v>2</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24"/>
-      <c r="L9" s="24"/>
-      <c r="M9" s="24">
+      <c r="C9" s="26"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23">
         <f t="shared" ref="M9:M10" si="1">L9*5</f>
         <v>0</v>
       </c>
-      <c r="N9" s="24"/>
-      <c r="O9" s="24"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="25">
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24">
         <f t="shared" ref="Q9:Q10" si="2">P9*N9</f>
         <v>0</v>
       </c>
-      <c r="R9" s="24"/>
-      <c r="S9" s="24"/>
-    </row>
-    <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R9" s="23"/>
+    </row>
+    <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="20">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C10" s="28"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -1246,9 +1106,8 @@
         <v>0</v>
       </c>
       <c r="R10" s="16"/>
-      <c r="S10" s="16"/>
-    </row>
-    <row r="11" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1262,19 +1121,18 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
-      <c r="N11" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="O11" s="48"/>
-      <c r="P11" s="48"/>
+      <c r="N11" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="O11" s="47"/>
+      <c r="P11" s="47"/>
       <c r="Q11" s="21" t="e">
         <f>SUM(#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
-    </row>
-    <row r="12" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1288,30 +1146,27 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="O12" s="48"/>
-      <c r="P12" s="48"/>
+      <c r="N12" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="O12" s="47"/>
+      <c r="P12" s="47"/>
       <c r="Q12" s="22" t="e">
         <f>Q11/5</f>
         <v>#REF!</v>
       </c>
       <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
     </row>
     <row r="24" spans="13:13" x14ac:dyDescent="0.25">
-      <c r="M24" s="44"/>
+      <c r="M24" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="K1:S1"/>
+  <mergeCells count="3">
+    <mergeCell ref="K1:R1"/>
     <mergeCell ref="N11:P11"/>
     <mergeCell ref="N12:P12"/>
-    <mergeCell ref="S2:S6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>